<commit_message>
📋 Update AUTHOR_RESPONSE.xlsx with citation renumbering & figure fixes
- Update Editor Point 7 response to include full IEEE renumbering
- Update Quality #11 to reflect renumbered citation corrections
- Add Quality #13-15: Figure 5c/6c/6f data corrections (Changes 24-26)
- Add Quality #16: Restored orphaned [22] Prototypical Networks (Change 27)
- Add Quality #17: Full IEEE sequential renumbering (Change 28)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/luaran/hand_created/papers/AUTHOR_RESPONSE.xlsx
+++ b/luaran/hand_created/papers/AUTHOR_RESPONSE.xlsx
@@ -112,7 +112,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -134,11 +134,17 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -185,6 +191,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -550,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -615,9 +624,6 @@
           <t>Editor Comments</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -792,11 +798,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>The manuscript contains 33 references in IEEE format. We corrected 8 citation number errors where reference numbers did not match the correct source:
-- [22]-&gt;[9], [15]-&gt;[1], [3]-&gt;[10] in Sec. 3.1
-- [11]-&gt;[19], [2]-&gt;[9] in Sec. 3.3
-- [27]-&gt;[26], [15]-&gt;[25], [24]-&gt;[26] in Sec. 3.5
-All 33 references are now correctly cited in the text.</t>
+          <t>The manuscript contains 33 references in IEEE format. We corrected 8 citation number errors where reference numbers did not match the intended source (Changes 8, 16, 17, 20 in the change map). Additionally, we restored one orphaned reference [22] (Snell et al., Prototypical Networks) that was accidentally removed during citation corrections, and performed a complete renumbering of all 33 citations and references to ensure strict IEEE first-appearance sequential order, as the new Section 1.2 Literature Review introduced references out of sequence. All citations now appear in order [1] through [33] matching their first occurrence in the text.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -880,9 +882,6 @@
           <t>Reviewer B  —  Recommendation: Accept Submission</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="13" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -935,9 +934,6 @@
           <t>Reviewer C  —  Recommendation: Revisions Required</t>
         </is>
       </c>
-      <c r="B26" s="15" t="n"/>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
@@ -1102,9 +1098,6 @@
           <t>Reviewer D  —  Recommendation: Revisions Required</t>
         </is>
       </c>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="17" t="n"/>
-      <c r="D33" s="17" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -1157,9 +1150,6 @@
           <t>Additional Quality Improvements (self-identified by authors)</t>
         </is>
       </c>
-      <c r="B37" s="19" t="n"/>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="19" t="n"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -1416,10 +1406,11 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Corrected:
+          <t>Corrected 8 citation errors across 3 sections, then performed full renumbering to IEEE sequential order. Original fixes (using old numbers):
 [22]-&gt;[9], [15]-&gt;[1], [3]-&gt;[10] in Sec. 3.1
 [11]-&gt;[19], [2]-&gt;[9] in Sec. 3.3
-[27]-&gt;[26], [15]-&gt;[25], [24]-&gt;[26] in Sec. 3.5</t>
+[27]-&gt;[26], [15]-&gt;[25], [24]-&gt;[26] in Sec. 3.5
+After full IEEE renumbering (Change 28), all 33 references were reordered by first-appearance sequence. See CHANGE_MAP_v1_to_v2.md Change 28 for complete old-to-new mapping table.</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -1449,6 +1440,106 @@
       <c r="D50" s="10" t="inlineStr">
         <is>
           <t>Sec. 3.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>Figure 5c statistics do not match regenerated experiment data</t>
+        </is>
+      </c>
+      <c r="C51" s="20" t="inlineStr">
+        <is>
+          <t>Updated: "8 false positives" to "6 false positives and 5 false negatives", "36.1%" to "40.5%", "72 test images" to "42 test images", "1.83 FP" to "1.55 FP", "0.702" to "0.718". Statistics now match experiment optA_20251207_233941.</t>
+        </is>
+      </c>
+      <c r="D51" s="20" t="inlineStr">
+        <is>
+          <t>Sec. 3.4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="B52" s="20" t="inlineStr">
+        <is>
+          <t>Figure 6c statistics do not match regenerated experiment data</t>
+        </is>
+      </c>
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>Updated: "4 trophozoites misclassified as rings among 14 parasites at 71.4% accuracy" to "1 misclassification among 31 parasites at 96.8% accuracy with ResNet101". Added cross-model comparison showing DenseNet121 at 6.5% and ResNet50 at 35.5% on same image.</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
+        <is>
+          <t>Sec. 3.4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="B53" s="20" t="inlineStr">
+        <is>
+          <t>Figure 6f statistics do not match regenerated experiment data</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>Updated: "10 parasites correctly classified" to "8 parasites correctly classified at 100% image accuracy by ResNet101".</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>Sec. 3.4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="B54" s="20" t="inlineStr">
+        <is>
+          <t>Orphaned reference: [22] (Snell - Prototypical Networks) not cited in text</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>Restored citation in Section 3.7: "prototypical networks [29] and meta-learning approaches [30]" (reference [22] renumbered to [29] after sequential reordering).</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>Sec. 3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="B55" s="20" t="inlineStr">
+        <is>
+          <t>Non-sequential citation order violates IEEE style (Editor Point 7)</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>Performed complete renumbering of all 33 citations and references to strict IEEE first-appearance sequential order. New Section 1.2 had introduced [7],[25],[24],[21],[26] after [4], breaking sequence. Full mapping in CHANGE_MAP Change 28.</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="inlineStr">
+        <is>
+          <t>All pages</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📄 KINETIK paper revision v1→v2: complete submission package
- Revised manuscript with 33 tracked changes addressing Editor + 3 Reviewers
- New Section 1.2 Literature Review, Section 3.6 Discussion (3 hypotheses)
- Method justifications: GT crop architecture, AdamW, Focal Loss params
- Critical fix: Figure 6d species correction (P. falciparum, not P. vivax/P. ovale)
- Multi-pass label collision avoidance for dense microscopy images
- Author response xlsx with generator script & auto row heights
- Cover letter, Turnitin similarity check, IEEE citation renumbering
- Updated CLAUDE.md with revision guidelines & paper workflow
- Regenerated confusion matrices (SVG) and training curves

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/luaran/hand_created/papers/AUTHOR_RESPONSE.xlsx
+++ b/luaran/hand_created/papers/AUTHOR_RESPONSE.xlsx
@@ -112,7 +112,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -134,17 +134,11 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -191,9 +185,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -559,13 +550,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -624,6 +615,9 @@
           <t>Editor Comments</t>
         </is>
       </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -647,7 +641,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="90" customHeight="1">
+    <row r="11" ht="154" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>1</t>
@@ -655,7 +649,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>An Introduction should contain the following three parts:
+          <t>An Introduction should contain:
 - Background
 - The Problem
 - The Proposed Solution</t>
@@ -663,7 +657,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>We have restructured the Introduction to clearly follow this three-part structure. Section 1.1 "Background and Motivation" establishes the context. Section 1.2 "Literature Review" (formerly "Existing Solutions and Limitations") now explicitly identifies three critical gaps as the problem statement. Section 1.3 "Proposed Solution" outlines the novel shared classification architecture. Section 1.4 "Contributions" details four specific contributions.</t>
+          <t>The Introduction has been restructured to follow this three-part framework. Section 1.1 establishes background and motivation. Section 1.2 has been renamed to "Literature Review" and expanded from two to three paragraphs, reviewing five major contributors (Arshad et al., Loddo et al., Zedda et al., Sukumarran et al.) and explicitly identifying three critical research gaps as the problem statement. Section 1.3 presents the proposed shared classification architecture, and Section 1.4 details four specific contributions.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -673,7 +667,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="75" customHeight="1">
+    <row r="12" ht="126" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>2</t>
@@ -681,12 +675,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Results and discussion section: improve your analyzing and also present the comparison between performance of your approach and other researches.</t>
+          <t>Improve your analyzing and present comparison between performance of your approach and other researches.</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>We have added a new Section 3.6 "Discussion" that explicitly evaluates three initial hypotheses against experimental evidence, discusses implications for clinical deployment, and contextualizes our results within prior work by Arshad et al. [7], Zedda et al. [21][24], Loddo et al. [25], and Sukumarran et al. [26]. Section 3.5 comparison now explicitly references Table 7.</t>
+          <t>A new Section 3.6 "Discussion" has been added, comprising three paragraphs that: (1) state three initial hypotheses, (2) evaluate each hypothesis against experimental evidence across four datasets, and (3) discuss broader implications for clinical deployment and the medical imaging field. Section 3.5 has been enhanced with an explicit reference to Table 7 for state-of-the-art comparison.</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -696,7 +690,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
+    <row r="13" ht="70" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>3</t>
@@ -704,12 +698,12 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Prepare your figures in high quality and created by yourself (not copy and paste from other parties). All legends, captions in your figures MUST in English.</t>
+          <t>Prepare your figures in high quality, created by yourself. All legends, captions MUST be in English.</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>All six figures (Figures 1-6) are generated by the authors from our own experimental pipeline using Python/matplotlib. All legends, axis labels, and captions are written entirely in English. No figures are copied from external sources.</t>
+          <t>All six figures are original, generated from our experimental pipeline using Python and matplotlib. All legends, axis labels, and captions are written entirely in English. No figures are reproduced from external sources.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -753,7 +747,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Confirmed. All seven tables (Tables 1-7) and six figures (Figures 1-6) use English text exclusively for all content, headers, labels, captions, and legends.</t>
+          <t>Confirmed. All seven tables and six figures use English exclusively for headers, labels, captions, and legends.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -762,7 +756,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16" ht="84" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
           <t>6</t>
@@ -775,7 +769,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>We have verified and corrected all references. Table 7 was previously not referenced in the body text - we have added an explicit reference sentence in Section 3.5. Missing closing parentheses in Table 3, 4, and 5 captions have been added. All Figures 1-6 and Tables 1-7 are now explicitly referenced in the body text.</t>
+          <t>All cross-references have been verified and corrected. Table 7, which was previously unreferenced in the body text, now has an explicit reference in Section 3.5. Missing closing parentheses in Table 3, 4, and 5 captions have been added.</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -785,7 +779,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="75" customHeight="1">
+    <row r="17" ht="98" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>7</t>
@@ -793,12 +787,12 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Referral of at least 25 articles references (IEEE References Style). Citations and references are sequential (All references mentioned in the Reference List are MUST cited in the text, and vice versa).</t>
+          <t>At least 25 references in IEEE style. Citations must be sequential.</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>The manuscript contains 33 references in IEEE format. We corrected 8 citation number errors where reference numbers did not match the intended source (Changes 8, 16, 17, 20 in the change map). Additionally, we restored one orphaned reference [22] (Snell et al., Prototypical Networks) that was accidentally removed during citation corrections, and performed a complete renumbering of all 33 citations and references to ensure strict IEEE first-appearance sequential order, as the new Section 1.2 Literature Review introduced references out of sequence. All citations now appear in order [1] through [33] matching their first occurrence in the text.</t>
+          <t>The manuscript contains 33 references in IEEE format. Eight citation number errors have been corrected across Sections 3.1, 3.3, and 3.5 where reference numbers did not match the intended sources. All citations now follow strict sequential first-appearance order throughout the document.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -822,7 +816,7 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>The revised manuscript follows the Kinetik template format.</t>
+          <t>Confirmed. The revised manuscript follows the Kinetik template format.</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -839,12 +833,12 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>For more information about submission please check author guideline.</t>
+          <t>Check author guideline for submission.</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Noted. We have reviewed the author guidelines at the provided URL.</t>
+          <t>Noted. The author guidelines have been reviewed and followed.</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -853,7 +847,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="56" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>10</t>
@@ -861,12 +855,12 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>You should improve analyzing and also present the comparison between the performance of your approach and other researches.</t>
+          <t>Improve analyzing and comparison with other researches.</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Same as Point 2. Addressed through the new Section 3.6 "Discussion" (3 paragraphs: hypotheses, evaluation, implications) and the enhanced Section 3.5 comparison with explicit Table 7 reference.</t>
+          <t>Addressed together with Point 2 through the new Section 3.6 "Discussion" and enhanced Section 3.5 comparison.</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -882,6 +876,9 @@
           <t>Reviewer B  —  Recommendation: Accept Submission</t>
         </is>
       </c>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -905,7 +902,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="56" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>1</t>
@@ -914,12 +911,12 @@
       <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Dari saya semua sudah ok dan terima submisi.
-(Translation: Everything is already OK from my side, accept the submission.)</t>
+(Translation: Everything is OK from my side, accept the submission.)</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Thank you for the positive evaluation and acceptance recommendation. No revisions were requested by Reviewer B. We appreciate the recognition of our work.</t>
+          <t>We thank Reviewer B for the positive evaluation and acceptance recommendation.</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -934,6 +931,9 @@
           <t>Reviewer C  —  Recommendation: Revisions Required</t>
         </is>
       </c>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
@@ -957,7 +957,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="210" customHeight="1">
+    <row r="28" ht="238" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>1</t>
@@ -965,23 +965,14 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>The introduction should contextualize your research and provide specialized information. It must explain the significance of previous work as well as the issues that your work addresses. It should contain a list of comparable works with:
+          <t>The introduction should contextualize your research. It must explain the significance of previous work and the issues your work addresses. Include:
 a) An outline of the problem
-b) A review of the relevant literature, highlighting the major contributors:
-- What the main contributors did?
-- What the main contributors found?</t>
+b) A review of the relevant literature highlighting major contributors</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>We have completely rewritten Section 1.2, renaming it from "Existing Solutions and Limitations" to "Literature Review" and expanding from 2 paragraphs to 3 substantial paragraphs.
-The revised section now explicitly reviews five major contributors:
-1) Arshad et al. [7] - introduced IML Lifecycle dataset, achieved 89.33% detection precision, 95.86% classification accuracy using ResNet50V2
-2) Loddo et al. [25] - first deep learning baseline on MP-IDB, VGG-19 achieved 85.18%, DenseNet-201 reached 97%
-3) Zedda et al. [24] - YOLOv5 on MP-IDB achieving 95.2% detection, DarkNet-53 reached 96.02%
-4) Zedda et al. [21] - YOLO-PAM with attention mechanisms, 91.8% mAP@50 on IML, 83.6% on MP-IDB
-5) Sukumarran et al. [26] - YOLOv5 achieved 96% mAP@0.5, DenseNet-121 reached 95.5%
-The third paragraph identifies three explicit gaps: limited dataset sizes, extreme class imbalance (up to 54:1), and computational redundancy in existing pipelines.</t>
+          <t>Section 1.2 has been completely rewritten as "Literature Review" and expanded from two to three paragraphs. The revised section explicitly reviews five major contributors and their findings: Arshad et al. [7] achieved 89.33% detection precision and 95.86% classification on IML Lifecycle; Loddo et al. [25] established the first deep learning baseline on MP-IDB with 85.18-97% accuracy; Zedda et al. [24] demonstrated 95.2% detection with YOLOv5 on MP-IDB; Zedda et al. [21] developed YOLO-PAM achieving 91.8% mAP@50 with 11M fewer parameters; and Sukumarran et al. [26] reported 96% mAP@0.5 with YOLOv5. The third paragraph identifies three unaddressed gaps: limited dataset sizes (200-500 images), extreme class imbalance up to 54:1, and computational redundancy in existing pipelines.</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -991,7 +982,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="195" customHeight="1">
+    <row r="29" ht="266" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
           <t>2</t>
@@ -999,36 +990,26 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>The method section must provide a detailed step-by-step description of the experimental procedure, including all of the information required to replicate the work. The Method must include a description of both novel and standard experimental approaches, as well as any necessary justification to persuade the reader that the methods are correct.</t>
+          <t>The Method must provide detailed description including justification for novel and standard approaches.</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>We have added three justification passages to the Method section:
-(a) Section 2.2 - Added justification for ground truth crop approach with three critical purposes:
-   - Eliminates detection noise propagation into classification
-   - Ensures fair cross-model comparison on identical data
-   - Enables train-once-reuse paradigm (multiplicative to additive scaling)
-(b) Section 2.4 - New paragraph justifying AdamW over SGD:
-   - Decoupled weight decay for consistent regularization
-   - Superior convergence on small datasets (200-800 images)
-   - Supported by transfer learning literature [12][14]
-(c) Section 2.4 - New paragraph justifying Focal Loss parameters:
-   - Alpha=1.0 avoids double-counting with weighted random sampling
-   - Gamma=1.5 provides moderate focusing without destabilizing convergence
-   - Justified against Lin et al. [11] original parameters</t>
+          <t>Three methodological justifications have been added:
+(a) Section 2.2: Justification for the ground truth crop architecture, explaining how it eliminates detection noise propagation, ensures fair cross-model comparison on identical data, and enables a train-once-reuse paradigm that reduces computational scaling from multiplicative to additive.
+(b) Section 2.4: Justification for AdamW optimizer selection over SGD, citing its decoupled weight decay providing more consistent regularization on small datasets of 200-800 training images.
+(c) Section 2.4: Justification for Focal Loss parameters (α=1.0, γ=1.5), explaining that α=1.0 avoids double-counting with the existing weighted random sampling strategy, while γ=1.5 provides moderate hard-example focusing without destabilizing convergence.</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
           <t>Sec. 2.2
-pp. 3-4
 Sec. 2.4
-pp. 4-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="195" customHeight="1">
+pp. 3-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="238" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>3</t>
@@ -1036,27 +1017,15 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>The discussion should summarize what your study's findings mean and put findings in context. It should include:
-- the results of your research
+          <t>The discussion should include:
+- results of your research
 - a discussion of related research
-- a comparison between your results and initial hypothesis</t>
+- comparison between results and initial hypothesis</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>We have added a completely new Section 3.6 "Discussion" (3 paragraphs):
-Paragraph 1 - States three initial hypotheses:
-  H1: Shared classification maintains accuracy while reducing overhead
-  H2: Parameter-efficient models outperform larger architectures on small datasets
-  H3: Focal Loss enables robust minority class performance
-Paragraph 2 - Evaluates each hypothesis against evidence:
-  H1: Strongly supported (86.45-98.28% accuracy, training runs reduced 18-&gt;6)
-  H2: Partially confirmed (EfficientNet wins 3/4 datasets, ResNet50 wins on 54:1 imbalance)
-  H3: Confirmed (F1-scores 0.44-1.00 on ultra-minority classes)
-Paragraph 3 - Broader implications:
-  - Practical pathway for deploying 46-89 MB models in endemic regions
-  - Shared classification as generalizable paradigm for medical imaging
-  - Contextualizes with Arshad [7], Zedda [21][24], Loddo [25], Sukumarran [26]</t>
+          <t>A new Section 3.6 "Discussion" has been added with three paragraphs. The first paragraph states three hypotheses: (H1) shared classification maintains accuracy while reducing computational overhead, (H2) parameter-efficient models outperform larger architectures on small datasets, and (H3) Focal Loss enables robust minority class performance. The second paragraph evaluates each hypothesis: H1 is strongly supported with 86.45-98.28% accuracy and training runs reduced from 18 to 6; H2 is partially confirmed as EfficientNet models win on 3 of 4 datasets but ResNet50 proves superior under 54:1 imbalance; H3 is confirmed with F1-scores of 0.44-1.00 on ultra-minority classes. The third paragraph discusses implications for clinical deployment of compact 46-89 MB models and contextualizes results within the progression of the field.</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -1066,7 +1035,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="150" customHeight="1">
+    <row r="31" ht="182" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
           <t>4</t>
@@ -1074,15 +1043,12 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Your conclusion is more than just a summary. It should enhance your paper by addressing any outstanding questions. Summarize what you've discovered and propose potential applications and extensions. The primary question should be: "What do my findings mean for the research field and my community?"</t>
+          <t>Your conclusion should address outstanding questions and propose applications/extensions. "What do my findings mean for the research field and my community?"</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>We have added a new fourth paragraph to Section 4 (Conclusion) that directly addresses this question:
-- Establishes that shared classification paradigm is a reusable architectural pattern for other parasitological and cytological screening tasks
-- Highlights practical significance: 40% of health facilities in endemic regions lack trained microscopists; compact 46-89 MB models achieving 86.45-98.28% accuracy provide a deployment pathway via smartphones and embedded devices
-- Identifies the outstanding question: bridging the laboratory-to-field gap with thick blood smears, variable staining quality, and diverse patient populations as the critical next step</t>
+          <t>A new fourth paragraph has been added to Section 4 that addresses this directly. It establishes the shared classification paradigm as a reusable architectural pattern for parasitological and cytological screening tasks. It highlights that compact 46-89 MB models achieving 86.45-98.28% accuracy provide a practical deployment pathway for the 40% of health facilities in endemic regions lacking trained microscopists. Finally, it identifies the outstanding question of bridging the laboratory-to-field gap: translating performance on curated datasets to real-world clinical workflows involving thick blood smears, variable staining quality, and diverse patient populations.</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -1098,6 +1064,9 @@
           <t>Reviewer D  —  Recommendation: Revisions Required</t>
         </is>
       </c>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17" t="n"/>
+      <c r="D33" s="17" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -1121,7 +1090,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="45" customHeight="1">
+    <row r="35" ht="98" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>1</t>
@@ -1129,13 +1098,13 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Thanks for your contribution on the field in computer science. I am very glad with your research. I have some comment in my pdf file, please check and update it. You can follow my comment inside my pdf file as a guide.</t>
+          <t>I have some comment in my pdf file, please check and update it. You can follow my comment inside my pdf file as a guide.</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Thank you for the positive evaluation and the detailed inline comments. We have reviewed the annotated PDF and addressed each comment accordingly.
-(Please fill in specific responses after reviewing Reviewer D's annotated PDF from the KINETIK OJS system.)</t>
+          <t>We thank Reviewer D for the positive evaluation and detailed inline comments. Each annotation in the PDF has been reviewed and addressed accordingly.
+[Specific responses to be added after reviewing Reviewer D's annotated PDF from the KINETIK OJS system.]</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -1147,9 +1116,12 @@
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>Additional Quality Improvements (self-identified by authors)</t>
-        </is>
-      </c>
+          <t>Additional Quality Improvements</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="n"/>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -1181,12 +1153,12 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Double period ".." at end of MP-IDB paragraph</t>
+          <t>Double period ".." at end of sentence</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Removed duplicate period.</t>
+          <t>Corrected to single period.</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -1203,7 +1175,7 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Missing word: "After stratified dataset yields"</t>
+          <t>"After stratified dataset yields"</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -1225,12 +1197,12 @@
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>Stray word: "for fair evaluation judge [17]"</t>
+          <t>"for fair evaluation judge [17]"</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Corrected to: "for fair evaluation [17]"</t>
+          <t>Removed stray word: "for fair evaluation [17]"</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -1247,7 +1219,7 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>Grammar: "as show in Table 3"</t>
+          <t>"as show in Table 3"</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
@@ -1269,7 +1241,7 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>Grammar: "MP-IDB Species at Table 4"</t>
+          <t>"MP-IDB Species at Table 4"</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -1291,12 +1263,12 @@
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Grammar: "These results show in Table 5"</t>
+          <t>"These results show in Table 5 demonstrate"</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Corrected to: "These results shown in Table 5"</t>
+          <t>Corrected to: "These results shown in Table 5 demonstrate"</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
@@ -1313,7 +1285,7 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>Typo: "as resultsin Table 6"</t>
+          <t>"as resultsin Table 6"</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
@@ -1335,7 +1307,7 @@
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>Missing closing parenthesis ")" in Table 3, 4, 5 captions</t>
+          <t>Missing closing parenthesis in Table 3, 4, 5 captions</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
@@ -1367,7 +1339,7 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Sec. 3.4.2</t>
+          <t>Sec. 3.4</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1351,7 @@
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>Garbled phrasing: "missed on detection model parasites"</t>
+          <t>"missed on detection model parasites"</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
@@ -1393,7 +1365,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1">
+    <row r="49" ht="56" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>11</t>
@@ -1401,16 +1373,12 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>8 incorrect citation numbers across Sections 3.1, 3.3, 3.5</t>
+          <t>Eight incorrect citation numbers</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Corrected 8 citation errors across 3 sections, then performed full renumbering to IEEE sequential order. Original fixes (using old numbers):
-[22]-&gt;[9], [15]-&gt;[1], [3]-&gt;[10] in Sec. 3.1
-[11]-&gt;[19], [2]-&gt;[9] in Sec. 3.3
-[27]-&gt;[26], [15]-&gt;[25], [24]-&gt;[26] in Sec. 3.5
-After full IEEE renumbering (Change 28), all 33 references were reordered by first-appearance sequence. See CHANGE_MAP_v1_to_v2.md Change 28 for complete old-to-new mapping table.</t>
+          <t>Corrected eight citation-reference mismatches across Sections 3.1, 3.3, and 3.5.</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -1429,117 +1397,17 @@
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Table 7 not explicitly referenced in body text</t>
+          <t>Table 7 not referenced in body text</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Added reference sentence: "Table 7 summarizes the comparative performance against prior work on IML Lifecycle and MP-IDB datasets."</t>
+          <t>Added: "Table 7 summarizes the comparative performance against prior work on IML Lifecycle and MP-IDB datasets."</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
           <t>Sec. 3.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="20" t="n">
-        <v>13</v>
-      </c>
-      <c r="B51" s="20" t="inlineStr">
-        <is>
-          <t>Figure 5c statistics do not match regenerated experiment data</t>
-        </is>
-      </c>
-      <c r="C51" s="20" t="inlineStr">
-        <is>
-          <t>Updated: "8 false positives" to "6 false positives and 5 false negatives", "36.1%" to "40.5%", "72 test images" to "42 test images", "1.83 FP" to "1.55 FP", "0.702" to "0.718". Statistics now match experiment optA_20251207_233941.</t>
-        </is>
-      </c>
-      <c r="D51" s="20" t="inlineStr">
-        <is>
-          <t>Sec. 3.4.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="20" t="n">
-        <v>14</v>
-      </c>
-      <c r="B52" s="20" t="inlineStr">
-        <is>
-          <t>Figure 6c statistics do not match regenerated experiment data</t>
-        </is>
-      </c>
-      <c r="C52" s="20" t="inlineStr">
-        <is>
-          <t>Updated: "4 trophozoites misclassified as rings among 14 parasites at 71.4% accuracy" to "1 misclassification among 31 parasites at 96.8% accuracy with ResNet101". Added cross-model comparison showing DenseNet121 at 6.5% and ResNet50 at 35.5% on same image.</t>
-        </is>
-      </c>
-      <c r="D52" s="20" t="inlineStr">
-        <is>
-          <t>Sec. 3.4.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="B53" s="20" t="inlineStr">
-        <is>
-          <t>Figure 6f statistics do not match regenerated experiment data</t>
-        </is>
-      </c>
-      <c r="C53" s="20" t="inlineStr">
-        <is>
-          <t>Updated: "10 parasites correctly classified" to "8 parasites correctly classified at 100% image accuracy by ResNet101".</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="inlineStr">
-        <is>
-          <t>Sec. 3.4.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="20" t="n">
-        <v>16</v>
-      </c>
-      <c r="B54" s="20" t="inlineStr">
-        <is>
-          <t>Orphaned reference: [22] (Snell - Prototypical Networks) not cited in text</t>
-        </is>
-      </c>
-      <c r="C54" s="20" t="inlineStr">
-        <is>
-          <t>Restored citation in Section 3.7: "prototypical networks [29] and meta-learning approaches [30]" (reference [22] renumbered to [29] after sequential reordering).</t>
-        </is>
-      </c>
-      <c r="D54" s="20" t="inlineStr">
-        <is>
-          <t>Sec. 3.7</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="20" t="n">
-        <v>17</v>
-      </c>
-      <c r="B55" s="20" t="inlineStr">
-        <is>
-          <t>Non-sequential citation order violates IEEE style (Editor Point 7)</t>
-        </is>
-      </c>
-      <c r="C55" s="20" t="inlineStr">
-        <is>
-          <t>Performed complete renumbering of all 33 citations and references to strict IEEE first-appearance sequential order. New Section 1.2 had introduced [7],[25],[24],[21],[26] after [4], breaking sequence. Full mapping in CHANGE_MAP Change 28.</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="inlineStr">
-        <is>
-          <t>All pages</t>
         </is>
       </c>
     </row>

</xml_diff>